<commit_message>
some updates to HIV catalog pages
</commit_message>
<xml_diff>
--- a/hiv/catalogo_HIV.xlsx
+++ b/hiv/catalogo_HIV.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N155"/>
+  <dimension ref="A1:O155"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -454,11 +454,12 @@
     <col width="30" customWidth="1" min="7" max="7"/>
     <col width="40" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="22" customWidth="1" min="12" max="12"/>
-    <col width="35" customWidth="1" min="13" max="13"/>
-    <col width="50" customWidth="1" min="14" max="14"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
+    <col width="35" customWidth="1" min="14" max="14"/>
+    <col width="50" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -509,25 +510,30 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
+          <t>Gastos em 2024 (USD)</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>Pop. elegível</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Cobertura</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Custo por unidade</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Notas</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>URL da Ficha</t>
         </is>
@@ -577,21 +583,26 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
+          <t>200.000</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
           <t>2.477.000</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>82.0%</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>0.09841212043675299</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr"/>
-      <c r="N2" s="2" t="inlineStr">
+      <c r="N2" s="2" t="inlineStr"/>
+      <c r="O2" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_01.html</t>
         </is>
@@ -643,11 +654,16 @@
           <t>2011</t>
         </is>
       </c>
-      <c r="J3" s="3" t="inlineStr"/>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K3" s="3" t="inlineStr"/>
       <c r="L3" s="3" t="inlineStr"/>
       <c r="M3" s="3" t="inlineStr"/>
-      <c r="N3" s="3" t="inlineStr">
+      <c r="N3" s="3" t="inlineStr"/>
+      <c r="O3" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_02.html</t>
         </is>
@@ -701,11 +717,16 @@
           <t>2011</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K4" s="2" t="inlineStr"/>
       <c r="L4" s="2" t="inlineStr"/>
       <c r="M4" s="2" t="inlineStr"/>
-      <c r="N4" s="2" t="inlineStr">
+      <c r="N4" s="2" t="inlineStr"/>
+      <c r="O4" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_03.html</t>
         </is>
@@ -753,11 +774,16 @@
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr"/>
-      <c r="J5" s="3" t="inlineStr"/>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K5" s="3" t="inlineStr"/>
       <c r="L5" s="3" t="inlineStr"/>
       <c r="M5" s="3" t="inlineStr"/>
-      <c r="N5" s="3" t="inlineStr">
+      <c r="N5" s="3" t="inlineStr"/>
+      <c r="O5" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_04.html</t>
         </is>
@@ -806,11 +832,16 @@
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr"/>
-      <c r="J6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K6" s="2" t="inlineStr"/>
       <c r="L6" s="2" t="inlineStr"/>
       <c r="M6" s="2" t="inlineStr"/>
-      <c r="N6" s="2" t="inlineStr">
+      <c r="N6" s="2" t="inlineStr"/>
+      <c r="O6" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_05.html</t>
         </is>
@@ -859,11 +890,16 @@
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr"/>
-      <c r="J7" s="3" t="inlineStr"/>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K7" s="3" t="inlineStr"/>
       <c r="L7" s="3" t="inlineStr"/>
       <c r="M7" s="3" t="inlineStr"/>
-      <c r="N7" s="3" t="inlineStr">
+      <c r="N7" s="3" t="inlineStr"/>
+      <c r="O7" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_06.html</t>
         </is>
@@ -911,11 +947,16 @@
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr"/>
-      <c r="J8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K8" s="2" t="inlineStr"/>
       <c r="L8" s="2" t="inlineStr"/>
       <c r="M8" s="2" t="inlineStr"/>
-      <c r="N8" s="2" t="inlineStr">
+      <c r="N8" s="2" t="inlineStr"/>
+      <c r="O8" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_07.html</t>
         </is>
@@ -963,11 +1004,16 @@
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr"/>
-      <c r="J9" s="3" t="inlineStr"/>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K9" s="3" t="inlineStr"/>
       <c r="L9" s="3" t="inlineStr"/>
       <c r="M9" s="3" t="inlineStr"/>
-      <c r="N9" s="3" t="inlineStr">
+      <c r="N9" s="3" t="inlineStr"/>
+      <c r="O9" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_08.html</t>
         </is>
@@ -1016,11 +1062,16 @@
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr"/>
-      <c r="J10" s="2" t="inlineStr"/>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K10" s="2" t="inlineStr"/>
       <c r="L10" s="2" t="inlineStr"/>
       <c r="M10" s="2" t="inlineStr"/>
-      <c r="N10" s="2" t="inlineStr">
+      <c r="N10" s="2" t="inlineStr"/>
+      <c r="O10" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_09.html</t>
         </is>
@@ -1069,11 +1120,16 @@
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr"/>
-      <c r="J11" s="3" t="inlineStr"/>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K11" s="3" t="inlineStr"/>
       <c r="L11" s="3" t="inlineStr"/>
       <c r="M11" s="3" t="inlineStr"/>
-      <c r="N11" s="3" t="inlineStr">
+      <c r="N11" s="3" t="inlineStr"/>
+      <c r="O11" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_10.html</t>
         </is>
@@ -1122,11 +1178,16 @@
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr"/>
-      <c r="J12" s="2" t="inlineStr"/>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K12" s="2" t="inlineStr"/>
       <c r="L12" s="2" t="inlineStr"/>
       <c r="M12" s="2" t="inlineStr"/>
-      <c r="N12" s="2" t="inlineStr">
+      <c r="N12" s="2" t="inlineStr"/>
+      <c r="O12" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_11.html</t>
         </is>
@@ -1175,11 +1236,16 @@
         </is>
       </c>
       <c r="I13" s="3" t="inlineStr"/>
-      <c r="J13" s="3" t="inlineStr"/>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K13" s="3" t="inlineStr"/>
       <c r="L13" s="3" t="inlineStr"/>
       <c r="M13" s="3" t="inlineStr"/>
-      <c r="N13" s="3" t="inlineStr">
+      <c r="N13" s="3" t="inlineStr"/>
+      <c r="O13" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_12.html</t>
         </is>
@@ -1228,11 +1294,16 @@
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr"/>
-      <c r="J14" s="2" t="inlineStr"/>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K14" s="2" t="inlineStr"/>
       <c r="L14" s="2" t="inlineStr"/>
       <c r="M14" s="2" t="inlineStr"/>
-      <c r="N14" s="2" t="inlineStr">
+      <c r="N14" s="2" t="inlineStr"/>
+      <c r="O14" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_13.html</t>
         </is>
@@ -1281,11 +1352,16 @@
         </is>
       </c>
       <c r="I15" s="3" t="inlineStr"/>
-      <c r="J15" s="3" t="inlineStr"/>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K15" s="3" t="inlineStr"/>
       <c r="L15" s="3" t="inlineStr"/>
       <c r="M15" s="3" t="inlineStr"/>
-      <c r="N15" s="3" t="inlineStr">
+      <c r="N15" s="3" t="inlineStr"/>
+      <c r="O15" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_14.html</t>
         </is>
@@ -1340,21 +1416,26 @@
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
+          <t>4.938.632</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
           <t>254.946</t>
         </is>
       </c>
-      <c r="K16" s="2" t="inlineStr">
+      <c r="L16" s="2" t="inlineStr">
         <is>
           <t>50.22630007782692</t>
         </is>
       </c>
-      <c r="L16" s="2" t="inlineStr">
+      <c r="M16" s="2" t="inlineStr">
         <is>
           <t>0.385679676495397</t>
         </is>
       </c>
-      <c r="M16" s="2" t="inlineStr"/>
-      <c r="N16" s="2" t="inlineStr">
+      <c r="N16" s="2" t="inlineStr"/>
+      <c r="O16" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_15.html</t>
         </is>
@@ -1409,21 +1490,26 @@
       </c>
       <c r="J17" s="3" t="inlineStr">
         <is>
+          <t>6.887.521</t>
+        </is>
+      </c>
+      <c r="K17" s="3" t="inlineStr">
+        <is>
           <t>254.946</t>
         </is>
       </c>
-      <c r="K17" s="3" t="inlineStr">
+      <c r="L17" s="3" t="inlineStr">
         <is>
           <t>50.22630007782692</t>
         </is>
       </c>
-      <c r="L17" s="3" t="inlineStr">
+      <c r="M17" s="3" t="inlineStr">
         <is>
           <t>0.537877067032586</t>
         </is>
       </c>
-      <c r="M17" s="3" t="inlineStr"/>
-      <c r="N17" s="3" t="inlineStr">
+      <c r="N17" s="3" t="inlineStr"/>
+      <c r="O17" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_16.html</t>
         </is>
@@ -1471,11 +1557,16 @@
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr"/>
-      <c r="J18" s="2" t="inlineStr"/>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K18" s="2" t="inlineStr"/>
       <c r="L18" s="2" t="inlineStr"/>
       <c r="M18" s="2" t="inlineStr"/>
-      <c r="N18" s="2" t="inlineStr">
+      <c r="N18" s="2" t="inlineStr"/>
+      <c r="O18" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_17.html</t>
         </is>
@@ -1523,11 +1614,16 @@
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr"/>
-      <c r="J19" s="3" t="inlineStr"/>
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K19" s="3" t="inlineStr"/>
       <c r="L19" s="3" t="inlineStr"/>
       <c r="M19" s="3" t="inlineStr"/>
-      <c r="N19" s="3" t="inlineStr">
+      <c r="N19" s="3" t="inlineStr"/>
+      <c r="O19" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_18.html</t>
         </is>
@@ -1576,11 +1672,16 @@
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr"/>
-      <c r="J20" s="2" t="inlineStr"/>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K20" s="2" t="inlineStr"/>
       <c r="L20" s="2" t="inlineStr"/>
       <c r="M20" s="2" t="inlineStr"/>
-      <c r="N20" s="2" t="inlineStr">
+      <c r="N20" s="2" t="inlineStr"/>
+      <c r="O20" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_19.html</t>
         </is>
@@ -1629,11 +1730,16 @@
         </is>
       </c>
       <c r="I21" s="3" t="inlineStr"/>
-      <c r="J21" s="3" t="inlineStr"/>
+      <c r="J21" s="3" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K21" s="3" t="inlineStr"/>
       <c r="L21" s="3" t="inlineStr"/>
       <c r="M21" s="3" t="inlineStr"/>
-      <c r="N21" s="3" t="inlineStr">
+      <c r="N21" s="3" t="inlineStr"/>
+      <c r="O21" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_20.html</t>
         </is>
@@ -1682,11 +1788,16 @@
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr"/>
-      <c r="J22" s="2" t="inlineStr"/>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K22" s="2" t="inlineStr"/>
       <c r="L22" s="2" t="inlineStr"/>
       <c r="M22" s="2" t="inlineStr"/>
-      <c r="N22" s="2" t="inlineStr">
+      <c r="N22" s="2" t="inlineStr"/>
+      <c r="O22" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_21.html</t>
         </is>
@@ -1734,11 +1845,16 @@
         </is>
       </c>
       <c r="I23" s="3" t="inlineStr"/>
-      <c r="J23" s="3" t="inlineStr"/>
+      <c r="J23" s="3" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K23" s="3" t="inlineStr"/>
       <c r="L23" s="3" t="inlineStr"/>
       <c r="M23" s="3" t="inlineStr"/>
-      <c r="N23" s="3" t="inlineStr">
+      <c r="N23" s="3" t="inlineStr"/>
+      <c r="O23" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_22.html</t>
         </is>
@@ -1786,11 +1902,16 @@
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr"/>
-      <c r="J24" s="2" t="inlineStr"/>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K24" s="2" t="inlineStr"/>
       <c r="L24" s="2" t="inlineStr"/>
       <c r="M24" s="2" t="inlineStr"/>
-      <c r="N24" s="2" t="inlineStr">
+      <c r="N24" s="2" t="inlineStr"/>
+      <c r="O24" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_23.html</t>
         </is>
@@ -1838,11 +1959,16 @@
         </is>
       </c>
       <c r="I25" s="3" t="inlineStr"/>
-      <c r="J25" s="3" t="inlineStr"/>
+      <c r="J25" s="3" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K25" s="3" t="inlineStr"/>
       <c r="L25" s="3" t="inlineStr"/>
       <c r="M25" s="3" t="inlineStr"/>
-      <c r="N25" s="3" t="inlineStr">
+      <c r="N25" s="3" t="inlineStr"/>
+      <c r="O25" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_24.html</t>
         </is>
@@ -1890,11 +2016,16 @@
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr"/>
-      <c r="J26" s="2" t="inlineStr"/>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K26" s="2" t="inlineStr"/>
       <c r="L26" s="2" t="inlineStr"/>
       <c r="M26" s="2" t="inlineStr"/>
-      <c r="N26" s="2" t="inlineStr">
+      <c r="N26" s="2" t="inlineStr"/>
+      <c r="O26" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_25.html</t>
         </is>
@@ -1942,11 +2073,16 @@
         </is>
       </c>
       <c r="I27" s="3" t="inlineStr"/>
-      <c r="J27" s="3" t="inlineStr"/>
+      <c r="J27" s="3" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K27" s="3" t="inlineStr"/>
       <c r="L27" s="3" t="inlineStr"/>
       <c r="M27" s="3" t="inlineStr"/>
-      <c r="N27" s="3" t="inlineStr">
+      <c r="N27" s="3" t="inlineStr"/>
+      <c r="O27" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_26.html</t>
         </is>
@@ -1994,11 +2130,16 @@
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr"/>
-      <c r="J28" s="2" t="inlineStr"/>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K28" s="2" t="inlineStr"/>
       <c r="L28" s="2" t="inlineStr"/>
       <c r="M28" s="2" t="inlineStr"/>
-      <c r="N28" s="2" t="inlineStr">
+      <c r="N28" s="2" t="inlineStr"/>
+      <c r="O28" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_27.html</t>
         </is>
@@ -2047,11 +2188,16 @@
         </is>
       </c>
       <c r="I29" s="3" t="inlineStr"/>
-      <c r="J29" s="3" t="inlineStr"/>
+      <c r="J29" s="3" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K29" s="3" t="inlineStr"/>
       <c r="L29" s="3" t="inlineStr"/>
       <c r="M29" s="3" t="inlineStr"/>
-      <c r="N29" s="3" t="inlineStr">
+      <c r="N29" s="3" t="inlineStr"/>
+      <c r="O29" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_28.html</t>
         </is>
@@ -2100,11 +2246,16 @@
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr"/>
-      <c r="J30" s="2" t="inlineStr"/>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K30" s="2" t="inlineStr"/>
       <c r="L30" s="2" t="inlineStr"/>
       <c r="M30" s="2" t="inlineStr"/>
-      <c r="N30" s="2" t="inlineStr">
+      <c r="N30" s="2" t="inlineStr"/>
+      <c r="O30" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_29.html</t>
         </is>
@@ -2153,11 +2304,16 @@
         </is>
       </c>
       <c r="I31" s="3" t="inlineStr"/>
-      <c r="J31" s="3" t="inlineStr"/>
+      <c r="J31" s="3" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K31" s="3" t="inlineStr"/>
       <c r="L31" s="3" t="inlineStr"/>
       <c r="M31" s="3" t="inlineStr"/>
-      <c r="N31" s="3" t="inlineStr">
+      <c r="N31" s="3" t="inlineStr"/>
+      <c r="O31" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_30.html</t>
         </is>
@@ -2206,11 +2362,16 @@
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr"/>
-      <c r="J32" s="2" t="inlineStr"/>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K32" s="2" t="inlineStr"/>
       <c r="L32" s="2" t="inlineStr"/>
       <c r="M32" s="2" t="inlineStr"/>
-      <c r="N32" s="2" t="inlineStr">
+      <c r="N32" s="2" t="inlineStr"/>
+      <c r="O32" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_31.html</t>
         </is>
@@ -2265,21 +2426,26 @@
       </c>
       <c r="J33" s="3" t="inlineStr">
         <is>
+          <t>61.567.205</t>
+        </is>
+      </c>
+      <c r="K33" s="3" t="inlineStr">
+        <is>
           <t>2.300.000</t>
         </is>
       </c>
-      <c r="K33" s="3" t="inlineStr">
+      <c r="L33" s="3" t="inlineStr">
         <is>
           <t>84.1%</t>
         </is>
       </c>
-      <c r="L33" s="3" t="inlineStr">
+      <c r="M33" s="3" t="inlineStr">
         <is>
           <t>31.82389388066507</t>
         </is>
       </c>
-      <c r="M33" s="3" t="inlineStr"/>
-      <c r="N33" s="3" t="inlineStr">
+      <c r="N33" s="3" t="inlineStr"/>
+      <c r="O33" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_32.html</t>
         </is>
@@ -2331,11 +2497,16 @@
           <t>2011</t>
         </is>
       </c>
-      <c r="J34" s="2" t="inlineStr"/>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K34" s="2" t="inlineStr"/>
       <c r="L34" s="2" t="inlineStr"/>
       <c r="M34" s="2" t="inlineStr"/>
-      <c r="N34" s="2" t="inlineStr">
+      <c r="N34" s="2" t="inlineStr"/>
+      <c r="O34" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_33.html</t>
         </is>
@@ -2387,11 +2558,16 @@
           <t>2011</t>
         </is>
       </c>
-      <c r="J35" s="3" t="inlineStr"/>
+      <c r="J35" s="3" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K35" s="3" t="inlineStr"/>
       <c r="L35" s="3" t="inlineStr"/>
       <c r="M35" s="3" t="inlineStr"/>
-      <c r="N35" s="3" t="inlineStr">
+      <c r="N35" s="3" t="inlineStr"/>
+      <c r="O35" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_34.html</t>
         </is>
@@ -2443,11 +2619,16 @@
           <t>Sem Informação</t>
         </is>
       </c>
-      <c r="J36" s="2" t="inlineStr"/>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K36" s="2" t="inlineStr"/>
       <c r="L36" s="2" t="inlineStr"/>
       <c r="M36" s="2" t="inlineStr"/>
-      <c r="N36" s="2" t="inlineStr">
+      <c r="N36" s="2" t="inlineStr"/>
+      <c r="O36" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_35.html</t>
         </is>
@@ -2495,11 +2676,16 @@
         </is>
       </c>
       <c r="I37" s="3" t="inlineStr"/>
-      <c r="J37" s="3" t="inlineStr"/>
+      <c r="J37" s="3" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K37" s="3" t="inlineStr"/>
       <c r="L37" s="3" t="inlineStr"/>
       <c r="M37" s="3" t="inlineStr"/>
-      <c r="N37" s="3" t="inlineStr">
+      <c r="N37" s="3" t="inlineStr"/>
+      <c r="O37" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_36.html</t>
         </is>
@@ -2548,11 +2734,16 @@
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr"/>
-      <c r="J38" s="2" t="inlineStr"/>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K38" s="2" t="inlineStr"/>
       <c r="L38" s="2" t="inlineStr"/>
       <c r="M38" s="2" t="inlineStr"/>
-      <c r="N38" s="2" t="inlineStr">
+      <c r="N38" s="2" t="inlineStr"/>
+      <c r="O38" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_37.html</t>
         </is>
@@ -2600,11 +2791,16 @@
         </is>
       </c>
       <c r="I39" s="3" t="inlineStr"/>
-      <c r="J39" s="3" t="inlineStr"/>
+      <c r="J39" s="3" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K39" s="3" t="inlineStr"/>
       <c r="L39" s="3" t="inlineStr"/>
       <c r="M39" s="3" t="inlineStr"/>
-      <c r="N39" s="3" t="inlineStr">
+      <c r="N39" s="3" t="inlineStr"/>
+      <c r="O39" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_38.html</t>
         </is>
@@ -2653,11 +2849,16 @@
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr"/>
-      <c r="J40" s="2" t="inlineStr"/>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K40" s="2" t="inlineStr"/>
       <c r="L40" s="2" t="inlineStr"/>
       <c r="M40" s="2" t="inlineStr"/>
-      <c r="N40" s="2" t="inlineStr">
+      <c r="N40" s="2" t="inlineStr"/>
+      <c r="O40" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_39.html</t>
         </is>
@@ -2705,11 +2906,16 @@
         </is>
       </c>
       <c r="I41" s="3" t="inlineStr"/>
-      <c r="J41" s="3" t="inlineStr"/>
+      <c r="J41" s="3" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K41" s="3" t="inlineStr"/>
       <c r="L41" s="3" t="inlineStr"/>
       <c r="M41" s="3" t="inlineStr"/>
-      <c r="N41" s="3" t="inlineStr">
+      <c r="N41" s="3" t="inlineStr"/>
+      <c r="O41" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_40.html</t>
         </is>
@@ -2757,11 +2963,16 @@
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr"/>
-      <c r="J42" s="2" t="inlineStr"/>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K42" s="2" t="inlineStr"/>
       <c r="L42" s="2" t="inlineStr"/>
       <c r="M42" s="2" t="inlineStr"/>
-      <c r="N42" s="2" t="inlineStr">
+      <c r="N42" s="2" t="inlineStr"/>
+      <c r="O42" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_41.html</t>
         </is>
@@ -2809,11 +3020,16 @@
         </is>
       </c>
       <c r="I43" s="3" t="inlineStr"/>
-      <c r="J43" s="3" t="inlineStr"/>
+      <c r="J43" s="3" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K43" s="3" t="inlineStr"/>
       <c r="L43" s="3" t="inlineStr"/>
       <c r="M43" s="3" t="inlineStr"/>
-      <c r="N43" s="3" t="inlineStr">
+      <c r="N43" s="3" t="inlineStr"/>
+      <c r="O43" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_42.html</t>
         </is>
@@ -2862,11 +3078,16 @@
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr"/>
-      <c r="J44" s="2" t="inlineStr"/>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K44" s="2" t="inlineStr"/>
       <c r="L44" s="2" t="inlineStr"/>
       <c r="M44" s="2" t="inlineStr"/>
-      <c r="N44" s="2" t="inlineStr">
+      <c r="N44" s="2" t="inlineStr"/>
+      <c r="O44" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_43.html</t>
         </is>
@@ -2914,11 +3135,16 @@
         </is>
       </c>
       <c r="I45" s="3" t="inlineStr"/>
-      <c r="J45" s="3" t="inlineStr"/>
+      <c r="J45" s="3" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K45" s="3" t="inlineStr"/>
       <c r="L45" s="3" t="inlineStr"/>
       <c r="M45" s="3" t="inlineStr"/>
-      <c r="N45" s="3" t="inlineStr">
+      <c r="N45" s="3" t="inlineStr"/>
+      <c r="O45" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_44.html</t>
         </is>
@@ -2967,11 +3193,16 @@
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr"/>
-      <c r="J46" s="2" t="inlineStr"/>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K46" s="2" t="inlineStr"/>
       <c r="L46" s="2" t="inlineStr"/>
       <c r="M46" s="2" t="inlineStr"/>
-      <c r="N46" s="2" t="inlineStr">
+      <c r="N46" s="2" t="inlineStr"/>
+      <c r="O46" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_45.html</t>
         </is>
@@ -3019,11 +3250,16 @@
         </is>
       </c>
       <c r="I47" s="3" t="inlineStr"/>
-      <c r="J47" s="3" t="inlineStr"/>
+      <c r="J47" s="3" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K47" s="3" t="inlineStr"/>
       <c r="L47" s="3" t="inlineStr"/>
       <c r="M47" s="3" t="inlineStr"/>
-      <c r="N47" s="3" t="inlineStr">
+      <c r="N47" s="3" t="inlineStr"/>
+      <c r="O47" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_46.html</t>
         </is>
@@ -3072,11 +3308,16 @@
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr"/>
-      <c r="J48" s="2" t="inlineStr"/>
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K48" s="2" t="inlineStr"/>
       <c r="L48" s="2" t="inlineStr"/>
       <c r="M48" s="2" t="inlineStr"/>
-      <c r="N48" s="2" t="inlineStr">
+      <c r="N48" s="2" t="inlineStr"/>
+      <c r="O48" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_47.html</t>
         </is>
@@ -3124,11 +3365,16 @@
         </is>
       </c>
       <c r="I49" s="3" t="inlineStr"/>
-      <c r="J49" s="3" t="inlineStr"/>
+      <c r="J49" s="3" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K49" s="3" t="inlineStr"/>
       <c r="L49" s="3" t="inlineStr"/>
       <c r="M49" s="3" t="inlineStr"/>
-      <c r="N49" s="3" t="inlineStr">
+      <c r="N49" s="3" t="inlineStr"/>
+      <c r="O49" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_48.html</t>
         </is>
@@ -3177,11 +3423,16 @@
         </is>
       </c>
       <c r="I50" s="2" t="inlineStr"/>
-      <c r="J50" s="2" t="inlineStr"/>
+      <c r="J50" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K50" s="2" t="inlineStr"/>
       <c r="L50" s="2" t="inlineStr"/>
       <c r="M50" s="2" t="inlineStr"/>
-      <c r="N50" s="2" t="inlineStr">
+      <c r="N50" s="2" t="inlineStr"/>
+      <c r="O50" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_49.html</t>
         </is>
@@ -3230,11 +3481,16 @@
         </is>
       </c>
       <c r="I51" s="3" t="inlineStr"/>
-      <c r="J51" s="3" t="inlineStr"/>
+      <c r="J51" s="3" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K51" s="3" t="inlineStr"/>
       <c r="L51" s="3" t="inlineStr"/>
       <c r="M51" s="3" t="inlineStr"/>
-      <c r="N51" s="3" t="inlineStr">
+      <c r="N51" s="3" t="inlineStr"/>
+      <c r="O51" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_50.html</t>
         </is>
@@ -3282,11 +3538,16 @@
         </is>
       </c>
       <c r="I52" s="2" t="inlineStr"/>
-      <c r="J52" s="2" t="inlineStr"/>
+      <c r="J52" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K52" s="2" t="inlineStr"/>
       <c r="L52" s="2" t="inlineStr"/>
       <c r="M52" s="2" t="inlineStr"/>
-      <c r="N52" s="2" t="inlineStr">
+      <c r="N52" s="2" t="inlineStr"/>
+      <c r="O52" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_51.html</t>
         </is>
@@ -3341,25 +3602,30 @@
       </c>
       <c r="J53" s="3" t="inlineStr">
         <is>
+          <t>3.850.406</t>
+        </is>
+      </c>
+      <c r="K53" s="3" t="inlineStr">
+        <is>
           <t>245.610</t>
         </is>
       </c>
-      <c r="K53" s="3" t="inlineStr">
+      <c r="L53" s="3" t="inlineStr">
         <is>
           <t>51.7%</t>
         </is>
       </c>
-      <c r="L53" s="3" t="inlineStr">
+      <c r="M53" s="3" t="inlineStr">
         <is>
           <t>30.33081522210056</t>
         </is>
       </c>
-      <c r="M53" s="3" t="inlineStr">
+      <c r="N53" s="3" t="inlineStr">
         <is>
           <t>Dados de SESP</t>
         </is>
       </c>
-      <c r="N53" s="3" t="inlineStr">
+      <c r="O53" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_52.html</t>
         </is>
@@ -3414,21 +3680,26 @@
       </c>
       <c r="J54" s="2" t="inlineStr">
         <is>
+          <t>4.007.197</t>
+        </is>
+      </c>
+      <c r="K54" s="2" t="inlineStr">
+        <is>
           <t>2.032.370</t>
         </is>
       </c>
-      <c r="K54" s="2" t="inlineStr">
+      <c r="L54" s="2" t="inlineStr">
         <is>
           <t>81.1%</t>
         </is>
       </c>
-      <c r="L54" s="2" t="inlineStr">
+      <c r="M54" s="2" t="inlineStr">
         <is>
           <t>2.430270082098699</t>
         </is>
       </c>
-      <c r="M54" s="2" t="inlineStr"/>
-      <c r="N54" s="2" t="inlineStr">
+      <c r="N54" s="2" t="inlineStr"/>
+      <c r="O54" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_53.html</t>
         </is>
@@ -3483,21 +3754,26 @@
       </c>
       <c r="J55" s="3" t="inlineStr">
         <is>
+          <t>3.993.859</t>
+        </is>
+      </c>
+      <c r="K55" s="3" t="inlineStr">
+        <is>
           <t>177.000</t>
         </is>
       </c>
-      <c r="K55" s="3" t="inlineStr">
+      <c r="L55" s="3" t="inlineStr">
         <is>
           <t>55.2%</t>
         </is>
       </c>
-      <c r="L55" s="3" t="inlineStr">
+      <c r="M55" s="3" t="inlineStr">
         <is>
           <t>40.8587316200843</t>
         </is>
       </c>
-      <c r="M55" s="3" t="inlineStr"/>
-      <c r="N55" s="3" t="inlineStr">
+      <c r="N55" s="3" t="inlineStr"/>
+      <c r="O55" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_54.html</t>
         </is>
@@ -3550,11 +3826,16 @@
           <t>2011</t>
         </is>
       </c>
-      <c r="J56" s="2" t="inlineStr"/>
+      <c r="J56" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K56" s="2" t="inlineStr"/>
       <c r="L56" s="2" t="inlineStr"/>
       <c r="M56" s="2" t="inlineStr"/>
-      <c r="N56" s="2" t="inlineStr">
+      <c r="N56" s="2" t="inlineStr"/>
+      <c r="O56" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_55.html</t>
         </is>
@@ -3607,11 +3888,16 @@
           <t>2011</t>
         </is>
       </c>
-      <c r="J57" s="3" t="inlineStr"/>
+      <c r="J57" s="3" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K57" s="3" t="inlineStr"/>
       <c r="L57" s="3" t="inlineStr"/>
       <c r="M57" s="3" t="inlineStr"/>
-      <c r="N57" s="3" t="inlineStr">
+      <c r="N57" s="3" t="inlineStr"/>
+      <c r="O57" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_56.html</t>
         </is>
@@ -3659,11 +3945,16 @@
         </is>
       </c>
       <c r="I58" s="2" t="inlineStr"/>
-      <c r="J58" s="2" t="inlineStr"/>
+      <c r="J58" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K58" s="2" t="inlineStr"/>
       <c r="L58" s="2" t="inlineStr"/>
       <c r="M58" s="2" t="inlineStr"/>
-      <c r="N58" s="2" t="inlineStr">
+      <c r="N58" s="2" t="inlineStr"/>
+      <c r="O58" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_57.html</t>
         </is>
@@ -3711,11 +4002,16 @@
         </is>
       </c>
       <c r="I59" s="3" t="inlineStr"/>
-      <c r="J59" s="3" t="inlineStr"/>
+      <c r="J59" s="3" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K59" s="3" t="inlineStr"/>
       <c r="L59" s="3" t="inlineStr"/>
       <c r="M59" s="3" t="inlineStr"/>
-      <c r="N59" s="3" t="inlineStr">
+      <c r="N59" s="3" t="inlineStr"/>
+      <c r="O59" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_58.html</t>
         </is>
@@ -3764,11 +4060,16 @@
         </is>
       </c>
       <c r="I60" s="2" t="inlineStr"/>
-      <c r="J60" s="2" t="inlineStr"/>
+      <c r="J60" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K60" s="2" t="inlineStr"/>
       <c r="L60" s="2" t="inlineStr"/>
       <c r="M60" s="2" t="inlineStr"/>
-      <c r="N60" s="2" t="inlineStr">
+      <c r="N60" s="2" t="inlineStr"/>
+      <c r="O60" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_59.html</t>
         </is>
@@ -3816,11 +4117,16 @@
         </is>
       </c>
       <c r="I61" s="3" t="inlineStr"/>
-      <c r="J61" s="3" t="inlineStr"/>
+      <c r="J61" s="3" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K61" s="3" t="inlineStr"/>
       <c r="L61" s="3" t="inlineStr"/>
       <c r="M61" s="3" t="inlineStr"/>
-      <c r="N61" s="3" t="inlineStr">
+      <c r="N61" s="3" t="inlineStr"/>
+      <c r="O61" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_60.html</t>
         </is>
@@ -3868,11 +4174,16 @@
         </is>
       </c>
       <c r="I62" s="2" t="inlineStr"/>
-      <c r="J62" s="2" t="inlineStr"/>
+      <c r="J62" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K62" s="2" t="inlineStr"/>
       <c r="L62" s="2" t="inlineStr"/>
       <c r="M62" s="2" t="inlineStr"/>
-      <c r="N62" s="2" t="inlineStr">
+      <c r="N62" s="2" t="inlineStr"/>
+      <c r="O62" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_61.html</t>
         </is>
@@ -3920,11 +4231,16 @@
         </is>
       </c>
       <c r="I63" s="3" t="inlineStr"/>
-      <c r="J63" s="3" t="inlineStr"/>
+      <c r="J63" s="3" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K63" s="3" t="inlineStr"/>
       <c r="L63" s="3" t="inlineStr"/>
       <c r="M63" s="3" t="inlineStr"/>
-      <c r="N63" s="3" t="inlineStr">
+      <c r="N63" s="3" t="inlineStr"/>
+      <c r="O63" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_62.html</t>
         </is>
@@ -3979,23 +4295,28 @@
       </c>
       <c r="J64" s="2" t="inlineStr">
         <is>
+          <t>509.142</t>
+        </is>
+      </c>
+      <c r="K64" s="2" t="inlineStr">
+        <is>
           <t>158.532</t>
         </is>
       </c>
-      <c r="K64" s="2" t="inlineStr">
+      <c r="L64" s="2" t="inlineStr">
         <is>
           <t>15.2%</t>
         </is>
       </c>
-      <c r="L64" s="2" t="e">
+      <c r="M64" s="2" t="e">
         <v>#VALUE!</v>
       </c>
-      <c r="M64" s="2" t="inlineStr">
+      <c r="N64" s="2" t="inlineStr">
         <is>
           <t>264541 novos inicios e 175826 reinicios</t>
         </is>
       </c>
-      <c r="N64" s="2" t="inlineStr">
+      <c r="O64" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_63.html</t>
         </is>
@@ -4050,17 +4371,22 @@
       </c>
       <c r="J65" s="3" t="inlineStr">
         <is>
+          <t>752.995</t>
+        </is>
+      </c>
+      <c r="K65" s="3" t="inlineStr">
+        <is>
           <t>158.532</t>
         </is>
       </c>
-      <c r="K65" s="3" t="inlineStr">
+      <c r="L65" s="3" t="inlineStr">
         <is>
           <t>15.2%</t>
         </is>
       </c>
-      <c r="L65" s="3" t="inlineStr"/>
       <c r="M65" s="3" t="inlineStr"/>
-      <c r="N65" s="3" t="inlineStr">
+      <c r="N65" s="3" t="inlineStr"/>
+      <c r="O65" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_64.html</t>
         </is>
@@ -4115,17 +4441,22 @@
       </c>
       <c r="J66" s="2" t="inlineStr">
         <is>
+          <t>2.000.618</t>
+        </is>
+      </c>
+      <c r="K66" s="2" t="inlineStr">
+        <is>
           <t>158.532</t>
         </is>
       </c>
-      <c r="K66" s="2" t="inlineStr">
+      <c r="L66" s="2" t="inlineStr">
         <is>
           <t>15.2%</t>
         </is>
       </c>
-      <c r="L66" s="2" t="inlineStr"/>
       <c r="M66" s="2" t="inlineStr"/>
-      <c r="N66" s="2" t="inlineStr">
+      <c r="N66" s="2" t="inlineStr"/>
+      <c r="O66" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_65.html</t>
         </is>
@@ -4174,11 +4505,16 @@
         </is>
       </c>
       <c r="I67" s="3" t="inlineStr"/>
-      <c r="J67" s="3" t="inlineStr"/>
+      <c r="J67" s="3" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K67" s="3" t="inlineStr"/>
       <c r="L67" s="3" t="inlineStr"/>
       <c r="M67" s="3" t="inlineStr"/>
-      <c r="N67" s="3" t="inlineStr">
+      <c r="N67" s="3" t="inlineStr"/>
+      <c r="O67" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_66.html</t>
         </is>
@@ -4227,11 +4563,16 @@
         </is>
       </c>
       <c r="I68" s="2" t="inlineStr"/>
-      <c r="J68" s="2" t="inlineStr"/>
+      <c r="J68" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K68" s="2" t="inlineStr"/>
       <c r="L68" s="2" t="inlineStr"/>
       <c r="M68" s="2" t="inlineStr"/>
-      <c r="N68" s="2" t="inlineStr">
+      <c r="N68" s="2" t="inlineStr"/>
+      <c r="O68" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_67.html</t>
         </is>
@@ -4280,11 +4621,16 @@
         </is>
       </c>
       <c r="I69" s="3" t="inlineStr"/>
-      <c r="J69" s="3" t="inlineStr"/>
+      <c r="J69" s="3" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K69" s="3" t="inlineStr"/>
       <c r="L69" s="3" t="inlineStr"/>
       <c r="M69" s="3" t="inlineStr"/>
-      <c r="N69" s="3" t="inlineStr">
+      <c r="N69" s="3" t="inlineStr"/>
+      <c r="O69" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_68.html</t>
         </is>
@@ -4333,11 +4679,16 @@
         </is>
       </c>
       <c r="I70" s="2" t="inlineStr"/>
-      <c r="J70" s="2" t="inlineStr"/>
+      <c r="J70" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K70" s="2" t="inlineStr"/>
       <c r="L70" s="2" t="inlineStr"/>
       <c r="M70" s="2" t="inlineStr"/>
-      <c r="N70" s="2" t="inlineStr">
+      <c r="N70" s="2" t="inlineStr"/>
+      <c r="O70" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_69.html</t>
         </is>
@@ -4386,11 +4737,16 @@
         </is>
       </c>
       <c r="I71" s="3" t="inlineStr"/>
-      <c r="J71" s="3" t="inlineStr"/>
+      <c r="J71" s="3" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K71" s="3" t="inlineStr"/>
       <c r="L71" s="3" t="inlineStr"/>
       <c r="M71" s="3" t="inlineStr"/>
-      <c r="N71" s="3" t="inlineStr">
+      <c r="N71" s="3" t="inlineStr"/>
+      <c r="O71" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_70.html</t>
         </is>
@@ -4439,11 +4795,16 @@
         </is>
       </c>
       <c r="I72" s="2" t="inlineStr"/>
-      <c r="J72" s="2" t="inlineStr"/>
+      <c r="J72" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K72" s="2" t="inlineStr"/>
       <c r="L72" s="2" t="inlineStr"/>
       <c r="M72" s="2" t="inlineStr"/>
-      <c r="N72" s="2" t="inlineStr">
+      <c r="N72" s="2" t="inlineStr"/>
+      <c r="O72" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_71.html</t>
         </is>
@@ -4492,11 +4853,16 @@
         </is>
       </c>
       <c r="I73" s="3" t="inlineStr"/>
-      <c r="J73" s="3" t="inlineStr"/>
+      <c r="J73" s="3" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K73" s="3" t="inlineStr"/>
       <c r="L73" s="3" t="inlineStr"/>
       <c r="M73" s="3" t="inlineStr"/>
-      <c r="N73" s="3" t="inlineStr">
+      <c r="N73" s="3" t="inlineStr"/>
+      <c r="O73" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_72.html</t>
         </is>
@@ -4544,11 +4910,16 @@
         </is>
       </c>
       <c r="I74" s="2" t="inlineStr"/>
-      <c r="J74" s="2" t="inlineStr"/>
+      <c r="J74" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K74" s="2" t="inlineStr"/>
       <c r="L74" s="2" t="inlineStr"/>
       <c r="M74" s="2" t="inlineStr"/>
-      <c r="N74" s="2" t="inlineStr">
+      <c r="N74" s="2" t="inlineStr"/>
+      <c r="O74" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_73.html</t>
         </is>
@@ -4596,11 +4967,16 @@
         </is>
       </c>
       <c r="I75" s="3" t="inlineStr"/>
-      <c r="J75" s="3" t="inlineStr"/>
+      <c r="J75" s="3" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K75" s="3" t="inlineStr"/>
       <c r="L75" s="3" t="inlineStr"/>
       <c r="M75" s="3" t="inlineStr"/>
-      <c r="N75" s="3" t="inlineStr">
+      <c r="N75" s="3" t="inlineStr"/>
+      <c r="O75" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_74.html</t>
         </is>
@@ -4649,11 +5025,16 @@
         </is>
       </c>
       <c r="I76" s="2" t="inlineStr"/>
-      <c r="J76" s="2" t="inlineStr"/>
+      <c r="J76" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K76" s="2" t="inlineStr"/>
       <c r="L76" s="2" t="inlineStr"/>
       <c r="M76" s="2" t="inlineStr"/>
-      <c r="N76" s="2" t="inlineStr">
+      <c r="N76" s="2" t="inlineStr"/>
+      <c r="O76" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_75.html</t>
         </is>
@@ -4702,11 +5083,16 @@
         </is>
       </c>
       <c r="I77" s="3" t="inlineStr"/>
-      <c r="J77" s="3" t="inlineStr"/>
+      <c r="J77" s="3" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K77" s="3" t="inlineStr"/>
       <c r="L77" s="3" t="inlineStr"/>
       <c r="M77" s="3" t="inlineStr"/>
-      <c r="N77" s="3" t="inlineStr">
+      <c r="N77" s="3" t="inlineStr"/>
+      <c r="O77" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_76.html</t>
         </is>
@@ -4755,11 +5141,16 @@
         </is>
       </c>
       <c r="I78" s="2" t="inlineStr"/>
-      <c r="J78" s="2" t="inlineStr"/>
+      <c r="J78" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K78" s="2" t="inlineStr"/>
       <c r="L78" s="2" t="inlineStr"/>
       <c r="M78" s="2" t="inlineStr"/>
-      <c r="N78" s="2" t="inlineStr">
+      <c r="N78" s="2" t="inlineStr"/>
+      <c r="O78" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_77.html</t>
         </is>
@@ -4808,11 +5199,16 @@
         </is>
       </c>
       <c r="I79" s="3" t="inlineStr"/>
-      <c r="J79" s="3" t="inlineStr"/>
+      <c r="J79" s="3" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K79" s="3" t="inlineStr"/>
       <c r="L79" s="3" t="inlineStr"/>
       <c r="M79" s="3" t="inlineStr"/>
-      <c r="N79" s="3" t="inlineStr">
+      <c r="N79" s="3" t="inlineStr"/>
+      <c r="O79" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_78.html</t>
         </is>
@@ -4861,11 +5257,16 @@
         </is>
       </c>
       <c r="I80" s="2" t="inlineStr"/>
-      <c r="J80" s="2" t="inlineStr"/>
+      <c r="J80" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K80" s="2" t="inlineStr"/>
       <c r="L80" s="2" t="inlineStr"/>
       <c r="M80" s="2" t="inlineStr"/>
-      <c r="N80" s="2" t="inlineStr">
+      <c r="N80" s="2" t="inlineStr"/>
+      <c r="O80" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_79.html</t>
         </is>
@@ -4914,11 +5315,16 @@
         </is>
       </c>
       <c r="I81" s="3" t="inlineStr"/>
-      <c r="J81" s="3" t="inlineStr"/>
+      <c r="J81" s="3" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K81" s="3" t="inlineStr"/>
       <c r="L81" s="3" t="inlineStr"/>
       <c r="M81" s="3" t="inlineStr"/>
-      <c r="N81" s="3" t="inlineStr">
+      <c r="N81" s="3" t="inlineStr"/>
+      <c r="O81" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_80.html</t>
         </is>
@@ -4967,11 +5373,16 @@
         </is>
       </c>
       <c r="I82" s="2" t="inlineStr"/>
-      <c r="J82" s="2" t="inlineStr"/>
+      <c r="J82" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K82" s="2" t="inlineStr"/>
       <c r="L82" s="2" t="inlineStr"/>
       <c r="M82" s="2" t="inlineStr"/>
-      <c r="N82" s="2" t="inlineStr">
+      <c r="N82" s="2" t="inlineStr"/>
+      <c r="O82" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_81.html</t>
         </is>
@@ -5020,11 +5431,16 @@
         </is>
       </c>
       <c r="I83" s="3" t="inlineStr"/>
-      <c r="J83" s="3" t="inlineStr"/>
+      <c r="J83" s="3" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K83" s="3" t="inlineStr"/>
       <c r="L83" s="3" t="inlineStr"/>
       <c r="M83" s="3" t="inlineStr"/>
-      <c r="N83" s="3" t="inlineStr">
+      <c r="N83" s="3" t="inlineStr"/>
+      <c r="O83" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_82.html</t>
         </is>
@@ -5073,11 +5489,16 @@
         </is>
       </c>
       <c r="I84" s="2" t="inlineStr"/>
-      <c r="J84" s="2" t="inlineStr"/>
+      <c r="J84" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K84" s="2" t="inlineStr"/>
       <c r="L84" s="2" t="inlineStr"/>
       <c r="M84" s="2" t="inlineStr"/>
-      <c r="N84" s="2" t="inlineStr">
+      <c r="N84" s="2" t="inlineStr"/>
+      <c r="O84" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_83.html</t>
         </is>
@@ -5125,11 +5546,16 @@
         </is>
       </c>
       <c r="I85" s="3" t="inlineStr"/>
-      <c r="J85" s="3" t="inlineStr"/>
+      <c r="J85" s="3" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K85" s="3" t="inlineStr"/>
       <c r="L85" s="3" t="inlineStr"/>
       <c r="M85" s="3" t="inlineStr"/>
-      <c r="N85" s="3" t="inlineStr">
+      <c r="N85" s="3" t="inlineStr"/>
+      <c r="O85" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_84.html</t>
         </is>
@@ -5177,11 +5603,16 @@
         </is>
       </c>
       <c r="I86" s="2" t="inlineStr"/>
-      <c r="J86" s="2" t="inlineStr"/>
+      <c r="J86" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K86" s="2" t="inlineStr"/>
       <c r="L86" s="2" t="inlineStr"/>
       <c r="M86" s="2" t="inlineStr"/>
-      <c r="N86" s="2" t="inlineStr">
+      <c r="N86" s="2" t="inlineStr"/>
+      <c r="O86" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_85.html</t>
         </is>
@@ -5230,11 +5661,16 @@
         </is>
       </c>
       <c r="I87" s="3" t="inlineStr"/>
-      <c r="J87" s="3" t="inlineStr"/>
+      <c r="J87" s="3" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K87" s="3" t="inlineStr"/>
       <c r="L87" s="3" t="inlineStr"/>
       <c r="M87" s="3" t="inlineStr"/>
-      <c r="N87" s="3" t="inlineStr">
+      <c r="N87" s="3" t="inlineStr"/>
+      <c r="O87" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_86.html</t>
         </is>
@@ -5282,11 +5718,16 @@
         </is>
       </c>
       <c r="I88" s="2" t="inlineStr"/>
-      <c r="J88" s="2" t="inlineStr"/>
+      <c r="J88" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K88" s="2" t="inlineStr"/>
       <c r="L88" s="2" t="inlineStr"/>
       <c r="M88" s="2" t="inlineStr"/>
-      <c r="N88" s="2" t="inlineStr">
+      <c r="N88" s="2" t="inlineStr"/>
+      <c r="O88" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_87.html</t>
         </is>
@@ -5334,11 +5775,16 @@
         </is>
       </c>
       <c r="I89" s="3" t="inlineStr"/>
-      <c r="J89" s="3" t="inlineStr"/>
+      <c r="J89" s="3" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K89" s="3" t="inlineStr"/>
       <c r="L89" s="3" t="inlineStr"/>
       <c r="M89" s="3" t="inlineStr"/>
-      <c r="N89" s="3" t="inlineStr">
+      <c r="N89" s="3" t="inlineStr"/>
+      <c r="O89" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_88.html</t>
         </is>
@@ -5392,23 +5838,28 @@
       </c>
       <c r="J90" s="2" t="inlineStr">
         <is>
+          <t>249.000</t>
+        </is>
+      </c>
+      <c r="K90" s="2" t="inlineStr">
+        <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="K90" s="2" t="e">
+      <c r="L90" s="2" t="e">
         <v>#VALUE!</v>
       </c>
-      <c r="L90" s="2" t="inlineStr">
+      <c r="M90" s="2" t="inlineStr">
         <is>
           <t>3507.042253521127</t>
         </is>
       </c>
-      <c r="M90" s="2" t="inlineStr">
+      <c r="N90" s="2" t="inlineStr">
         <is>
           <t># alcancado sao Unidade Santiarias</t>
         </is>
       </c>
-      <c r="N90" s="2" t="inlineStr">
+      <c r="O90" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_89.html</t>
         </is>
@@ -5460,11 +5911,16 @@
           <t>2011</t>
         </is>
       </c>
-      <c r="J91" s="3" t="inlineStr"/>
+      <c r="J91" s="3" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K91" s="3" t="inlineStr"/>
       <c r="L91" s="3" t="inlineStr"/>
       <c r="M91" s="3" t="inlineStr"/>
-      <c r="N91" s="3" t="inlineStr">
+      <c r="N91" s="3" t="inlineStr"/>
+      <c r="O91" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_90.html</t>
         </is>
@@ -5517,11 +5973,16 @@
           <t>2011</t>
         </is>
       </c>
-      <c r="J92" s="2" t="inlineStr"/>
+      <c r="J92" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K92" s="2" t="inlineStr"/>
       <c r="L92" s="2" t="inlineStr"/>
       <c r="M92" s="2" t="inlineStr"/>
-      <c r="N92" s="2" t="inlineStr">
+      <c r="N92" s="2" t="inlineStr"/>
+      <c r="O92" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_91.html</t>
         </is>
@@ -5569,11 +6030,16 @@
         </is>
       </c>
       <c r="I93" s="3" t="inlineStr"/>
-      <c r="J93" s="3" t="inlineStr"/>
+      <c r="J93" s="3" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K93" s="3" t="inlineStr"/>
       <c r="L93" s="3" t="inlineStr"/>
       <c r="M93" s="3" t="inlineStr"/>
-      <c r="N93" s="3" t="inlineStr">
+      <c r="N93" s="3" t="inlineStr"/>
+      <c r="O93" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_92.html</t>
         </is>
@@ -5621,11 +6087,16 @@
         </is>
       </c>
       <c r="I94" s="2" t="inlineStr"/>
-      <c r="J94" s="2" t="inlineStr"/>
+      <c r="J94" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K94" s="2" t="inlineStr"/>
       <c r="L94" s="2" t="inlineStr"/>
       <c r="M94" s="2" t="inlineStr"/>
-      <c r="N94" s="2" t="inlineStr">
+      <c r="N94" s="2" t="inlineStr"/>
+      <c r="O94" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_93.html</t>
         </is>
@@ -5673,11 +6144,16 @@
         </is>
       </c>
       <c r="I95" s="3" t="inlineStr"/>
-      <c r="J95" s="3" t="inlineStr"/>
+      <c r="J95" s="3" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K95" s="3" t="inlineStr"/>
       <c r="L95" s="3" t="inlineStr"/>
       <c r="M95" s="3" t="inlineStr"/>
-      <c r="N95" s="3" t="inlineStr">
+      <c r="N95" s="3" t="inlineStr"/>
+      <c r="O95" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_94.html</t>
         </is>
@@ -5726,11 +6202,16 @@
         </is>
       </c>
       <c r="I96" s="2" t="inlineStr"/>
-      <c r="J96" s="2" t="inlineStr"/>
+      <c r="J96" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K96" s="2" t="inlineStr"/>
       <c r="L96" s="2" t="inlineStr"/>
       <c r="M96" s="2" t="inlineStr"/>
-      <c r="N96" s="2" t="inlineStr">
+      <c r="N96" s="2" t="inlineStr"/>
+      <c r="O96" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_95.html</t>
         </is>
@@ -5779,11 +6260,16 @@
         </is>
       </c>
       <c r="I97" s="3" t="inlineStr"/>
-      <c r="J97" s="3" t="inlineStr"/>
+      <c r="J97" s="3" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K97" s="3" t="inlineStr"/>
       <c r="L97" s="3" t="inlineStr"/>
       <c r="M97" s="3" t="inlineStr"/>
-      <c r="N97" s="3" t="inlineStr">
+      <c r="N97" s="3" t="inlineStr"/>
+      <c r="O97" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_96.html</t>
         </is>
@@ -5832,11 +6318,16 @@
         </is>
       </c>
       <c r="I98" s="2" t="inlineStr"/>
-      <c r="J98" s="2" t="inlineStr"/>
+      <c r="J98" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K98" s="2" t="inlineStr"/>
       <c r="L98" s="2" t="inlineStr"/>
       <c r="M98" s="2" t="inlineStr"/>
-      <c r="N98" s="2" t="inlineStr">
+      <c r="N98" s="2" t="inlineStr"/>
+      <c r="O98" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_97.html</t>
         </is>
@@ -5885,11 +6376,16 @@
         </is>
       </c>
       <c r="I99" s="3" t="inlineStr"/>
-      <c r="J99" s="3" t="inlineStr"/>
+      <c r="J99" s="3" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K99" s="3" t="inlineStr"/>
       <c r="L99" s="3" t="inlineStr"/>
       <c r="M99" s="3" t="inlineStr"/>
-      <c r="N99" s="3" t="inlineStr">
+      <c r="N99" s="3" t="inlineStr"/>
+      <c r="O99" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_98.html</t>
         </is>
@@ -5938,11 +6434,16 @@
         </is>
       </c>
       <c r="I100" s="2" t="inlineStr"/>
-      <c r="J100" s="2" t="inlineStr"/>
+      <c r="J100" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K100" s="2" t="inlineStr"/>
       <c r="L100" s="2" t="inlineStr"/>
       <c r="M100" s="2" t="inlineStr"/>
-      <c r="N100" s="2" t="inlineStr">
+      <c r="N100" s="2" t="inlineStr"/>
+      <c r="O100" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_99.html</t>
         </is>
@@ -5990,11 +6491,16 @@
         </is>
       </c>
       <c r="I101" s="3" t="inlineStr"/>
-      <c r="J101" s="3" t="inlineStr"/>
+      <c r="J101" s="3" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K101" s="3" t="inlineStr"/>
       <c r="L101" s="3" t="inlineStr"/>
       <c r="M101" s="3" t="inlineStr"/>
-      <c r="N101" s="3" t="inlineStr">
+      <c r="N101" s="3" t="inlineStr"/>
+      <c r="O101" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_100.html</t>
         </is>
@@ -6038,11 +6544,16 @@
         </is>
       </c>
       <c r="I102" s="2" t="inlineStr"/>
-      <c r="J102" s="2" t="inlineStr"/>
+      <c r="J102" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K102" s="2" t="inlineStr"/>
       <c r="L102" s="2" t="inlineStr"/>
       <c r="M102" s="2" t="inlineStr"/>
-      <c r="N102" s="2" t="inlineStr">
+      <c r="N102" s="2" t="inlineStr"/>
+      <c r="O102" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_101.html</t>
         </is>
@@ -6090,11 +6601,16 @@
         </is>
       </c>
       <c r="I103" s="3" t="inlineStr"/>
-      <c r="J103" s="3" t="inlineStr"/>
+      <c r="J103" s="3" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K103" s="3" t="inlineStr"/>
       <c r="L103" s="3" t="inlineStr"/>
       <c r="M103" s="3" t="inlineStr"/>
-      <c r="N103" s="3" t="inlineStr">
+      <c r="N103" s="3" t="inlineStr"/>
+      <c r="O103" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_102.html</t>
         </is>
@@ -6142,11 +6658,16 @@
         </is>
       </c>
       <c r="I104" s="2" t="inlineStr"/>
-      <c r="J104" s="2" t="inlineStr"/>
+      <c r="J104" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K104" s="2" t="inlineStr"/>
       <c r="L104" s="2" t="inlineStr"/>
       <c r="M104" s="2" t="inlineStr"/>
-      <c r="N104" s="2" t="inlineStr">
+      <c r="N104" s="2" t="inlineStr"/>
+      <c r="O104" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_103.html</t>
         </is>
@@ -6200,21 +6721,26 @@
       </c>
       <c r="J105" s="3" t="inlineStr">
         <is>
+          <t>250.000</t>
+        </is>
+      </c>
+      <c r="K105" s="3" t="inlineStr">
+        <is>
           <t>2.032.370</t>
         </is>
       </c>
-      <c r="K105" s="3" t="inlineStr">
+      <c r="L105" s="3" t="inlineStr">
         <is>
           <t>91.0%</t>
         </is>
       </c>
-      <c r="L105" s="3" t="inlineStr">
+      <c r="M105" s="3" t="inlineStr">
         <is>
           <t>0.1351748107687824</t>
         </is>
       </c>
-      <c r="M105" s="3" t="inlineStr"/>
-      <c r="N105" s="3" t="inlineStr">
+      <c r="N105" s="3" t="inlineStr"/>
+      <c r="O105" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_104.html</t>
         </is>
@@ -6263,11 +6789,16 @@
         </is>
       </c>
       <c r="I106" s="2" t="inlineStr"/>
-      <c r="J106" s="2" t="inlineStr"/>
+      <c r="J106" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K106" s="2" t="inlineStr"/>
       <c r="L106" s="2" t="inlineStr"/>
       <c r="M106" s="2" t="inlineStr"/>
-      <c r="N106" s="2" t="inlineStr">
+      <c r="N106" s="2" t="inlineStr"/>
+      <c r="O106" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_105.html</t>
         </is>
@@ -6313,11 +6844,16 @@
         </is>
       </c>
       <c r="I107" s="3" t="inlineStr"/>
-      <c r="J107" s="3" t="inlineStr"/>
+      <c r="J107" s="3" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K107" s="3" t="inlineStr"/>
       <c r="L107" s="3" t="inlineStr"/>
       <c r="M107" s="3" t="inlineStr"/>
-      <c r="N107" s="3" t="inlineStr">
+      <c r="N107" s="3" t="inlineStr"/>
+      <c r="O107" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_106.html</t>
         </is>
@@ -6361,11 +6897,16 @@
         </is>
       </c>
       <c r="I108" s="2" t="inlineStr"/>
-      <c r="J108" s="2" t="inlineStr"/>
+      <c r="J108" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K108" s="2" t="inlineStr"/>
       <c r="L108" s="2" t="inlineStr"/>
       <c r="M108" s="2" t="inlineStr"/>
-      <c r="N108" s="2" t="inlineStr">
+      <c r="N108" s="2" t="inlineStr"/>
+      <c r="O108" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_107.html</t>
         </is>
@@ -6410,11 +6951,16 @@
         </is>
       </c>
       <c r="I109" s="3" t="inlineStr"/>
-      <c r="J109" s="3" t="inlineStr"/>
+      <c r="J109" s="3" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K109" s="3" t="inlineStr"/>
       <c r="L109" s="3" t="inlineStr"/>
       <c r="M109" s="3" t="inlineStr"/>
-      <c r="N109" s="3" t="inlineStr">
+      <c r="N109" s="3" t="inlineStr"/>
+      <c r="O109" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_108.html</t>
         </is>
@@ -6459,11 +7005,16 @@
         </is>
       </c>
       <c r="I110" s="2" t="inlineStr"/>
-      <c r="J110" s="2" t="inlineStr"/>
+      <c r="J110" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K110" s="2" t="inlineStr"/>
       <c r="L110" s="2" t="inlineStr"/>
       <c r="M110" s="2" t="inlineStr"/>
-      <c r="N110" s="2" t="inlineStr">
+      <c r="N110" s="2" t="inlineStr"/>
+      <c r="O110" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_109.html</t>
         </is>
@@ -6508,11 +7059,16 @@
         </is>
       </c>
       <c r="I111" s="3" t="inlineStr"/>
-      <c r="J111" s="3" t="inlineStr"/>
+      <c r="J111" s="3" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K111" s="3" t="inlineStr"/>
       <c r="L111" s="3" t="inlineStr"/>
       <c r="M111" s="3" t="inlineStr"/>
-      <c r="N111" s="3" t="inlineStr">
+      <c r="N111" s="3" t="inlineStr"/>
+      <c r="O111" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_110.html</t>
         </is>
@@ -6557,11 +7113,16 @@
         </is>
       </c>
       <c r="I112" s="2" t="inlineStr"/>
-      <c r="J112" s="2" t="inlineStr"/>
+      <c r="J112" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K112" s="2" t="inlineStr"/>
       <c r="L112" s="2" t="inlineStr"/>
       <c r="M112" s="2" t="inlineStr"/>
-      <c r="N112" s="2" t="inlineStr">
+      <c r="N112" s="2" t="inlineStr"/>
+      <c r="O112" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_111.html</t>
         </is>
@@ -6611,11 +7172,16 @@
         </is>
       </c>
       <c r="I113" s="3" t="inlineStr"/>
-      <c r="J113" s="3" t="inlineStr"/>
+      <c r="J113" s="3" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K113" s="3" t="inlineStr"/>
       <c r="L113" s="3" t="inlineStr"/>
       <c r="M113" s="3" t="inlineStr"/>
-      <c r="N113" s="3" t="inlineStr">
+      <c r="N113" s="3" t="inlineStr"/>
+      <c r="O113" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_112.html</t>
         </is>
@@ -6664,11 +7230,16 @@
         </is>
       </c>
       <c r="I114" s="2" t="inlineStr"/>
-      <c r="J114" s="2" t="inlineStr"/>
+      <c r="J114" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K114" s="2" t="inlineStr"/>
       <c r="L114" s="2" t="inlineStr"/>
       <c r="M114" s="2" t="inlineStr"/>
-      <c r="N114" s="2" t="inlineStr">
+      <c r="N114" s="2" t="inlineStr"/>
+      <c r="O114" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_113.html</t>
         </is>
@@ -6717,11 +7288,16 @@
         </is>
       </c>
       <c r="I115" s="3" t="inlineStr"/>
-      <c r="J115" s="3" t="inlineStr"/>
+      <c r="J115" s="3" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K115" s="3" t="inlineStr"/>
       <c r="L115" s="3" t="inlineStr"/>
       <c r="M115" s="3" t="inlineStr"/>
-      <c r="N115" s="3" t="inlineStr">
+      <c r="N115" s="3" t="inlineStr"/>
+      <c r="O115" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_114.html</t>
         </is>
@@ -6773,11 +7349,16 @@
         </is>
       </c>
       <c r="I116" s="2" t="inlineStr"/>
-      <c r="J116" s="2" t="inlineStr"/>
+      <c r="J116" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K116" s="2" t="inlineStr"/>
       <c r="L116" s="2" t="inlineStr"/>
       <c r="M116" s="2" t="inlineStr"/>
-      <c r="N116" s="2" t="inlineStr">
+      <c r="N116" s="2" t="inlineStr"/>
+      <c r="O116" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_115.html</t>
         </is>
@@ -6832,23 +7413,28 @@
       </c>
       <c r="J117" s="3" t="inlineStr">
         <is>
+          <t>82.431</t>
+        </is>
+      </c>
+      <c r="K117" s="3" t="inlineStr">
+        <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="K117" s="3" t="e">
+      <c r="L117" s="3" t="e">
         <v>#VALUE!</v>
       </c>
-      <c r="L117" s="3" t="inlineStr">
+      <c r="M117" s="3" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="M117" s="3" t="inlineStr">
+      <c r="N117" s="3" t="inlineStr">
         <is>
           <t>Nao iniciou em 2024</t>
         </is>
       </c>
-      <c r="N117" s="3" t="inlineStr">
+      <c r="O117" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_116.html</t>
         </is>
@@ -6903,25 +7489,30 @@
       </c>
       <c r="J118" s="2" t="inlineStr">
         <is>
+          <t>133.754</t>
+        </is>
+      </c>
+      <c r="K118" s="2" t="inlineStr">
+        <is>
           <t>3.185.533</t>
         </is>
       </c>
-      <c r="K118" s="2" t="inlineStr">
+      <c r="L118" s="2" t="inlineStr">
         <is>
           <t>0.0%</t>
         </is>
       </c>
-      <c r="L118" s="2" t="inlineStr">
+      <c r="M118" s="2" t="inlineStr">
         <is>
           <t>3715.393500000001</t>
         </is>
       </c>
-      <c r="M118" s="2" t="inlineStr">
+      <c r="N118" s="2" t="inlineStr">
         <is>
           <t>36 RAMJ 15-24 em seguimento no ano 2024, pois foi o inicio do piloto</t>
         </is>
       </c>
-      <c r="N118" s="2" t="inlineStr">
+      <c r="O118" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_117.html</t>
         </is>
@@ -6974,23 +7565,28 @@
           <t>&lt;2015</t>
         </is>
       </c>
-      <c r="J119" s="3" t="e">
-        <v>#VALUE!</v>
+      <c r="J119" s="3" t="inlineStr">
+        <is>
+          <t>147.227</t>
+        </is>
       </c>
       <c r="K119" s="3" t="e">
         <v>#VALUE!</v>
       </c>
-      <c r="L119" s="3" t="inlineStr">
+      <c r="L119" s="3" t="e">
+        <v>#VALUE!</v>
+      </c>
+      <c r="M119" s="3" t="inlineStr">
         <is>
           <t>0.061678806032677</t>
         </is>
       </c>
-      <c r="M119" s="3" t="inlineStr">
+      <c r="N119" s="3" t="inlineStr">
         <is>
           <t>dados de distribucao, Hom + Mulh 15-49</t>
         </is>
       </c>
-      <c r="N119" s="3" t="inlineStr">
+      <c r="O119" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_118.html</t>
         </is>
@@ -7045,23 +7641,28 @@
       </c>
       <c r="J120" s="2" t="inlineStr">
         <is>
+          <t>665.169</t>
+        </is>
+      </c>
+      <c r="K120" s="2" t="inlineStr">
+        <is>
           <t>todos utentes na US</t>
         </is>
       </c>
-      <c r="K120" s="2" t="e">
+      <c r="L120" s="2" t="e">
         <v>#VALUE!</v>
       </c>
-      <c r="L120" s="2" t="inlineStr">
+      <c r="M120" s="2" t="inlineStr">
         <is>
           <t>0.6309392820691827</t>
         </is>
       </c>
-      <c r="M120" s="2" t="inlineStr">
+      <c r="N120" s="2" t="inlineStr">
         <is>
           <t>por causa de cobertura de livro de ITS não é possivel calcular um pop. Eligivel</t>
         </is>
       </c>
-      <c r="N120" s="2" t="inlineStr">
+      <c r="O120" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_119.html</t>
         </is>
@@ -7116,25 +7717,30 @@
       </c>
       <c r="J121" s="3" t="inlineStr">
         <is>
+          <t>2.579.520</t>
+        </is>
+      </c>
+      <c r="K121" s="3" t="inlineStr">
+        <is>
           <t>8.159.149</t>
         </is>
       </c>
-      <c r="K121" s="3" t="inlineStr">
+      <c r="L121" s="3" t="inlineStr">
         <is>
           <t>68.6%</t>
         </is>
       </c>
-      <c r="L121" s="3" t="inlineStr">
+      <c r="M121" s="3" t="inlineStr">
         <is>
           <t>0.4605463310123192</t>
         </is>
       </c>
-      <c r="M121" s="3" t="inlineStr">
+      <c r="N121" s="3" t="inlineStr">
         <is>
           <t>dados de distribucao Mulher 15 - 49 anos</t>
         </is>
       </c>
-      <c r="N121" s="3" t="inlineStr">
+      <c r="O121" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_120.html</t>
         </is>
@@ -7189,25 +7795,30 @@
       </c>
       <c r="J122" s="2" t="inlineStr">
         <is>
+          <t>5.527.092</t>
+        </is>
+      </c>
+      <c r="K122" s="2" t="inlineStr">
+        <is>
           <t>30.767.054</t>
         </is>
       </c>
-      <c r="K122" s="2" t="inlineStr">
+      <c r="L122" s="2" t="inlineStr">
         <is>
           <t>0.8%</t>
         </is>
       </c>
-      <c r="L122" s="2" t="inlineStr">
+      <c r="M122" s="2" t="inlineStr">
         <is>
           <t>21.33839519575633</t>
         </is>
       </c>
-      <c r="M122" s="2" t="inlineStr">
+      <c r="N122" s="2" t="inlineStr">
         <is>
           <t>Novo inicios a PrEP para o ano 2024</t>
         </is>
       </c>
-      <c r="N122" s="2" t="inlineStr">
+      <c r="O122" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_121.html</t>
         </is>
@@ -7262,25 +7873,30 @@
       </c>
       <c r="J123" s="3" t="inlineStr">
         <is>
+          <t>7.491.341</t>
+        </is>
+      </c>
+      <c r="K123" s="3" t="inlineStr">
+        <is>
           <t>7.388.905</t>
         </is>
       </c>
-      <c r="K123" s="3" t="inlineStr">
+      <c r="L123" s="3" t="inlineStr">
         <is>
           <t>21.810947630264565</t>
         </is>
       </c>
-      <c r="L123" s="3" t="inlineStr">
+      <c r="M123" s="3" t="inlineStr">
         <is>
           <t>0.04648415651820172</t>
         </is>
       </c>
-      <c r="M123" s="3" t="inlineStr">
+      <c r="N123" s="3" t="inlineStr">
         <is>
           <t>dados de distribucao Homen 15 - 49 anos</t>
         </is>
       </c>
-      <c r="N123" s="3" t="inlineStr">
+      <c r="O123" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_122.html</t>
         </is>
@@ -7332,11 +7948,16 @@
           <t>2011</t>
         </is>
       </c>
-      <c r="J124" s="2" t="inlineStr"/>
+      <c r="J124" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K124" s="2" t="inlineStr"/>
       <c r="L124" s="2" t="inlineStr"/>
       <c r="M124" s="2" t="inlineStr"/>
-      <c r="N124" s="2" t="inlineStr">
+      <c r="N124" s="2" t="inlineStr"/>
+      <c r="O124" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_123.html</t>
         </is>
@@ -7388,11 +8009,16 @@
           <t>2011</t>
         </is>
       </c>
-      <c r="J125" s="3" t="inlineStr"/>
+      <c r="J125" s="3" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K125" s="3" t="inlineStr"/>
       <c r="L125" s="3" t="inlineStr"/>
       <c r="M125" s="3" t="inlineStr"/>
-      <c r="N125" s="3" t="inlineStr">
+      <c r="N125" s="3" t="inlineStr"/>
+      <c r="O125" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_124.html</t>
         </is>
@@ -7440,11 +8066,16 @@
         </is>
       </c>
       <c r="I126" s="2" t="inlineStr"/>
-      <c r="J126" s="2" t="inlineStr"/>
+      <c r="J126" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K126" s="2" t="inlineStr"/>
       <c r="L126" s="2" t="inlineStr"/>
       <c r="M126" s="2" t="inlineStr"/>
-      <c r="N126" s="2" t="inlineStr">
+      <c r="N126" s="2" t="inlineStr"/>
+      <c r="O126" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_125.html</t>
         </is>
@@ -7493,11 +8124,16 @@
         </is>
       </c>
       <c r="I127" s="3" t="inlineStr"/>
-      <c r="J127" s="3" t="inlineStr"/>
+      <c r="J127" s="3" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K127" s="3" t="inlineStr"/>
       <c r="L127" s="3" t="inlineStr"/>
       <c r="M127" s="3" t="inlineStr"/>
-      <c r="N127" s="3" t="inlineStr">
+      <c r="N127" s="3" t="inlineStr"/>
+      <c r="O127" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_126.html</t>
         </is>
@@ -7546,11 +8182,16 @@
         </is>
       </c>
       <c r="I128" s="2" t="inlineStr"/>
-      <c r="J128" s="2" t="inlineStr"/>
+      <c r="J128" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K128" s="2" t="inlineStr"/>
       <c r="L128" s="2" t="inlineStr"/>
       <c r="M128" s="2" t="inlineStr"/>
-      <c r="N128" s="2" t="inlineStr">
+      <c r="N128" s="2" t="inlineStr"/>
+      <c r="O128" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_127.html</t>
         </is>
@@ -7599,11 +8240,16 @@
         </is>
       </c>
       <c r="I129" s="3" t="inlineStr"/>
-      <c r="J129" s="3" t="inlineStr"/>
+      <c r="J129" s="3" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K129" s="3" t="inlineStr"/>
       <c r="L129" s="3" t="inlineStr"/>
       <c r="M129" s="3" t="inlineStr"/>
-      <c r="N129" s="3" t="inlineStr">
+      <c r="N129" s="3" t="inlineStr"/>
+      <c r="O129" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_128.html</t>
         </is>
@@ -7652,11 +8298,16 @@
         </is>
       </c>
       <c r="I130" s="2" t="inlineStr"/>
-      <c r="J130" s="2" t="inlineStr"/>
+      <c r="J130" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K130" s="2" t="inlineStr"/>
       <c r="L130" s="2" t="inlineStr"/>
       <c r="M130" s="2" t="inlineStr"/>
-      <c r="N130" s="2" t="inlineStr">
+      <c r="N130" s="2" t="inlineStr"/>
+      <c r="O130" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_129.html</t>
         </is>
@@ -7705,11 +8356,16 @@
         </is>
       </c>
       <c r="I131" s="3" t="inlineStr"/>
-      <c r="J131" s="3" t="inlineStr"/>
+      <c r="J131" s="3" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K131" s="3" t="inlineStr"/>
       <c r="L131" s="3" t="inlineStr"/>
       <c r="M131" s="3" t="inlineStr"/>
-      <c r="N131" s="3" t="inlineStr">
+      <c r="N131" s="3" t="inlineStr"/>
+      <c r="O131" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_130.html</t>
         </is>
@@ -7757,11 +8413,16 @@
         </is>
       </c>
       <c r="I132" s="2" t="inlineStr"/>
-      <c r="J132" s="2" t="inlineStr"/>
+      <c r="J132" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K132" s="2" t="inlineStr"/>
       <c r="L132" s="2" t="inlineStr"/>
       <c r="M132" s="2" t="inlineStr"/>
-      <c r="N132" s="2" t="inlineStr">
+      <c r="N132" s="2" t="inlineStr"/>
+      <c r="O132" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_131.html</t>
         </is>
@@ -7809,11 +8470,16 @@
         </is>
       </c>
       <c r="I133" s="3" t="inlineStr"/>
-      <c r="J133" s="3" t="inlineStr"/>
+      <c r="J133" s="3" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K133" s="3" t="inlineStr"/>
       <c r="L133" s="3" t="inlineStr"/>
       <c r="M133" s="3" t="inlineStr"/>
-      <c r="N133" s="3" t="inlineStr">
+      <c r="N133" s="3" t="inlineStr"/>
+      <c r="O133" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_132.html</t>
         </is>
@@ -7868,23 +8534,28 @@
       </c>
       <c r="J134" s="2" t="inlineStr">
         <is>
+          <t>48.899</t>
+        </is>
+      </c>
+      <c r="K134" s="2" t="inlineStr">
+        <is>
           <t>36.171</t>
         </is>
       </c>
-      <c r="K134" s="2" t="inlineStr">
+      <c r="L134" s="2" t="inlineStr">
         <is>
           <t>0.0%</t>
         </is>
       </c>
-      <c r="L134" s="2" t="e">
+      <c r="M134" s="2" t="e">
         <v>#DIV/0!</v>
       </c>
-      <c r="M134" s="2" t="inlineStr">
+      <c r="N134" s="2" t="inlineStr">
         <is>
           <t>Carga Viral para VHB nao foi implmentado em 2024</t>
         </is>
       </c>
-      <c r="N134" s="2" t="inlineStr">
+      <c r="O134" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_133.html</t>
         </is>
@@ -7939,25 +8610,30 @@
       </c>
       <c r="J135" s="3" t="inlineStr">
         <is>
+          <t>469.080</t>
+        </is>
+      </c>
+      <c r="K135" s="3" t="inlineStr">
+        <is>
           <t>36.171</t>
         </is>
       </c>
-      <c r="K135" s="3" t="inlineStr">
+      <c r="L135" s="3" t="inlineStr">
         <is>
           <t>89.1%</t>
         </is>
       </c>
-      <c r="L135" s="3" t="inlineStr">
+      <c r="M135" s="3" t="inlineStr">
         <is>
           <t>14.55053042992741</t>
         </is>
       </c>
-      <c r="M135" s="3" t="inlineStr">
+      <c r="N135" s="3" t="inlineStr">
         <is>
           <t>Ainda foi um piloto ate o fim de 2024, em MC tinha 7,615, Nampula 18,706, Sofala 5,917</t>
         </is>
       </c>
-      <c r="N135" s="3" t="inlineStr">
+      <c r="O135" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_134.html</t>
         </is>
@@ -8012,23 +8688,28 @@
       </c>
       <c r="J136" s="2" t="inlineStr">
         <is>
+          <t>750.350</t>
+        </is>
+      </c>
+      <c r="K136" s="2" t="inlineStr">
+        <is>
           <t>Pessoas com sinais ou sintomas</t>
         </is>
       </c>
-      <c r="K136" s="2" t="e">
+      <c r="L136" s="2" t="e">
         <v>#VALUE!</v>
       </c>
-      <c r="L136" s="2" t="inlineStr">
+      <c r="M136" s="2" t="inlineStr">
         <is>
           <t>2.041635729911516</t>
         </is>
       </c>
-      <c r="M136" s="2" t="inlineStr">
+      <c r="N136" s="2" t="inlineStr">
         <is>
           <t>testados para Sifilis no livro de ITS</t>
         </is>
       </c>
-      <c r="N136" s="2" t="inlineStr">
+      <c r="O136" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_135.html</t>
         </is>
@@ -8083,25 +8764,30 @@
       </c>
       <c r="J137" s="3" t="inlineStr">
         <is>
+          <t>884.603</t>
+        </is>
+      </c>
+      <c r="K137" s="3" t="inlineStr">
+        <is>
           <t>134.000</t>
         </is>
       </c>
-      <c r="K137" s="3" t="inlineStr">
+      <c r="L137" s="3" t="inlineStr">
         <is>
           <t>81.8%</t>
         </is>
       </c>
-      <c r="L137" s="3" t="inlineStr">
+      <c r="M137" s="3" t="inlineStr">
         <is>
           <t>8.066636253214423</t>
         </is>
       </c>
-      <c r="M137" s="3" t="inlineStr">
+      <c r="N137" s="3" t="inlineStr">
         <is>
           <t>MG HIV+ na CPN</t>
         </is>
       </c>
-      <c r="N137" s="3" t="inlineStr">
+      <c r="O137" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_136.html</t>
         </is>
@@ -8156,21 +8842,26 @@
       </c>
       <c r="J138" s="2" t="inlineStr">
         <is>
+          <t>2.786.852</t>
+        </is>
+      </c>
+      <c r="K138" s="2" t="inlineStr">
+        <is>
           <t>2.111.754</t>
         </is>
       </c>
-      <c r="K138" s="2" t="inlineStr">
+      <c r="L138" s="2" t="inlineStr">
         <is>
           <t>99.0%</t>
         </is>
       </c>
-      <c r="L138" s="2" t="inlineStr">
+      <c r="M138" s="2" t="inlineStr">
         <is>
           <t>1.33270233448056</t>
         </is>
       </c>
-      <c r="M138" s="2" t="inlineStr"/>
-      <c r="N138" s="2" t="inlineStr">
+      <c r="N138" s="2" t="inlineStr"/>
+      <c r="O138" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_137.html</t>
         </is>
@@ -8222,11 +8913,16 @@
           <t>2011</t>
         </is>
       </c>
-      <c r="J139" s="3" t="inlineStr"/>
+      <c r="J139" s="3" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K139" s="3" t="inlineStr"/>
       <c r="L139" s="3" t="inlineStr"/>
       <c r="M139" s="3" t="inlineStr"/>
-      <c r="N139" s="3" t="inlineStr">
+      <c r="N139" s="3" t="inlineStr"/>
+      <c r="O139" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_138.html</t>
         </is>
@@ -8278,11 +8974,16 @@
           <t>2011</t>
         </is>
       </c>
-      <c r="J140" s="2" t="inlineStr"/>
+      <c r="J140" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K140" s="2" t="inlineStr"/>
       <c r="L140" s="2" t="inlineStr"/>
       <c r="M140" s="2" t="inlineStr"/>
-      <c r="N140" s="2" t="inlineStr">
+      <c r="N140" s="2" t="inlineStr"/>
+      <c r="O140" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_139.html</t>
         </is>
@@ -8336,17 +9037,22 @@
       </c>
       <c r="J141" s="3" t="inlineStr">
         <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
+      <c r="K141" s="3" t="inlineStr">
+        <is>
           <t>Mulher Lactante  e pacientes HIV+                                                                                                                                                                                  ESMI</t>
         </is>
       </c>
-      <c r="K141" s="3" t="inlineStr">
+      <c r="L141" s="3" t="inlineStr">
         <is>
           <t>Todas as US AJUDA (149) Manica (51), Niassa(18), Sofala (47) e Tete (33)</t>
         </is>
       </c>
-      <c r="L141" s="3" t="inlineStr"/>
       <c r="M141" s="3" t="inlineStr"/>
-      <c r="N141" s="3" t="inlineStr">
+      <c r="N141" s="3" t="inlineStr"/>
+      <c r="O141" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_140.html</t>
         </is>
@@ -8395,11 +9101,16 @@
         </is>
       </c>
       <c r="I142" s="2" t="inlineStr"/>
-      <c r="J142" s="2" t="inlineStr"/>
+      <c r="J142" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K142" s="2" t="inlineStr"/>
       <c r="L142" s="2" t="inlineStr"/>
       <c r="M142" s="2" t="inlineStr"/>
-      <c r="N142" s="2" t="inlineStr">
+      <c r="N142" s="2" t="inlineStr"/>
+      <c r="O142" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_141.html</t>
         </is>
@@ -8447,11 +9158,16 @@
         </is>
       </c>
       <c r="I143" s="3" t="inlineStr"/>
-      <c r="J143" s="3" t="inlineStr"/>
+      <c r="J143" s="3" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K143" s="3" t="inlineStr"/>
       <c r="L143" s="3" t="inlineStr"/>
       <c r="M143" s="3" t="inlineStr"/>
-      <c r="N143" s="3" t="inlineStr">
+      <c r="N143" s="3" t="inlineStr"/>
+      <c r="O143" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_142.html</t>
         </is>
@@ -8499,11 +9215,16 @@
         </is>
       </c>
       <c r="I144" s="2" t="inlineStr"/>
-      <c r="J144" s="2" t="inlineStr"/>
+      <c r="J144" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K144" s="2" t="inlineStr"/>
       <c r="L144" s="2" t="inlineStr"/>
       <c r="M144" s="2" t="inlineStr"/>
-      <c r="N144" s="2" t="inlineStr">
+      <c r="N144" s="2" t="inlineStr"/>
+      <c r="O144" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_143.html</t>
         </is>
@@ -8552,11 +9273,16 @@
         </is>
       </c>
       <c r="I145" s="3" t="inlineStr"/>
-      <c r="J145" s="3" t="inlineStr"/>
+      <c r="J145" s="3" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K145" s="3" t="inlineStr"/>
       <c r="L145" s="3" t="inlineStr"/>
       <c r="M145" s="3" t="inlineStr"/>
-      <c r="N145" s="3" t="inlineStr">
+      <c r="N145" s="3" t="inlineStr"/>
+      <c r="O145" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_144.html</t>
         </is>
@@ -8605,11 +9331,16 @@
         </is>
       </c>
       <c r="I146" s="2" t="inlineStr"/>
-      <c r="J146" s="2" t="inlineStr"/>
+      <c r="J146" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K146" s="2" t="inlineStr"/>
       <c r="L146" s="2" t="inlineStr"/>
       <c r="M146" s="2" t="inlineStr"/>
-      <c r="N146" s="2" t="inlineStr">
+      <c r="N146" s="2" t="inlineStr"/>
+      <c r="O146" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_145.html</t>
         </is>
@@ -8657,11 +9388,16 @@
         </is>
       </c>
       <c r="I147" s="3" t="inlineStr"/>
-      <c r="J147" s="3" t="inlineStr"/>
+      <c r="J147" s="3" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K147" s="3" t="inlineStr"/>
       <c r="L147" s="3" t="inlineStr"/>
       <c r="M147" s="3" t="inlineStr"/>
-      <c r="N147" s="3" t="inlineStr">
+      <c r="N147" s="3" t="inlineStr"/>
+      <c r="O147" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_146.html</t>
         </is>
@@ -8709,11 +9445,16 @@
         </is>
       </c>
       <c r="I148" s="2" t="inlineStr"/>
-      <c r="J148" s="2" t="inlineStr"/>
+      <c r="J148" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K148" s="2" t="inlineStr"/>
       <c r="L148" s="2" t="inlineStr"/>
       <c r="M148" s="2" t="inlineStr"/>
-      <c r="N148" s="2" t="inlineStr">
+      <c r="N148" s="2" t="inlineStr"/>
+      <c r="O148" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_147.html</t>
         </is>
@@ -8761,11 +9502,16 @@
         </is>
       </c>
       <c r="I149" s="3" t="inlineStr"/>
-      <c r="J149" s="3" t="inlineStr"/>
+      <c r="J149" s="3" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K149" s="3" t="inlineStr"/>
       <c r="L149" s="3" t="inlineStr"/>
       <c r="M149" s="3" t="inlineStr"/>
-      <c r="N149" s="3" t="inlineStr">
+      <c r="N149" s="3" t="inlineStr"/>
+      <c r="O149" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_148.html</t>
         </is>
@@ -8814,11 +9560,16 @@
         </is>
       </c>
       <c r="I150" s="2" t="inlineStr"/>
-      <c r="J150" s="2" t="inlineStr"/>
+      <c r="J150" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K150" s="2" t="inlineStr"/>
       <c r="L150" s="2" t="inlineStr"/>
       <c r="M150" s="2" t="inlineStr"/>
-      <c r="N150" s="2" t="inlineStr">
+      <c r="N150" s="2" t="inlineStr"/>
+      <c r="O150" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_149.html</t>
         </is>
@@ -8867,11 +9618,16 @@
         </is>
       </c>
       <c r="I151" s="3" t="inlineStr"/>
-      <c r="J151" s="3" t="inlineStr"/>
+      <c r="J151" s="3" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K151" s="3" t="inlineStr"/>
       <c r="L151" s="3" t="inlineStr"/>
       <c r="M151" s="3" t="inlineStr"/>
-      <c r="N151" s="3" t="inlineStr">
+      <c r="N151" s="3" t="inlineStr"/>
+      <c r="O151" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_150.html</t>
         </is>
@@ -8920,11 +9676,16 @@
         </is>
       </c>
       <c r="I152" s="2" t="inlineStr"/>
-      <c r="J152" s="2" t="inlineStr"/>
+      <c r="J152" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K152" s="2" t="inlineStr"/>
       <c r="L152" s="2" t="inlineStr"/>
       <c r="M152" s="2" t="inlineStr"/>
-      <c r="N152" s="2" t="inlineStr">
+      <c r="N152" s="2" t="inlineStr"/>
+      <c r="O152" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_151.html</t>
         </is>
@@ -8979,21 +9740,26 @@
       </c>
       <c r="J153" s="3" t="inlineStr">
         <is>
+          <t>3.674.196</t>
+        </is>
+      </c>
+      <c r="K153" s="3" t="inlineStr">
+        <is>
           <t>266.240</t>
         </is>
       </c>
-      <c r="K153" s="3" t="inlineStr">
+      <c r="L153" s="3" t="inlineStr">
         <is>
           <t>93.2%</t>
         </is>
       </c>
-      <c r="L153" s="3" t="inlineStr">
+      <c r="M153" s="3" t="inlineStr">
         <is>
           <t>14.80509942741094</t>
         </is>
       </c>
-      <c r="M153" s="3" t="inlineStr"/>
-      <c r="N153" s="3" t="inlineStr">
+      <c r="N153" s="3" t="inlineStr"/>
+      <c r="O153" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_152.html</t>
         </is>
@@ -9045,11 +9811,16 @@
           <t>2011</t>
         </is>
       </c>
-      <c r="J154" s="2" t="inlineStr"/>
+      <c r="J154" s="2" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K154" s="2" t="inlineStr"/>
       <c r="L154" s="2" t="inlineStr"/>
       <c r="M154" s="2" t="inlineStr"/>
-      <c r="N154" s="2" t="inlineStr">
+      <c r="N154" s="2" t="inlineStr"/>
+      <c r="O154" s="2" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_153.html</t>
         </is>
@@ -9101,11 +9872,16 @@
           <t>2011</t>
         </is>
       </c>
-      <c r="J155" s="3" t="inlineStr"/>
+      <c r="J155" s="3" t="inlineStr">
+        <is>
+          <t>Sem Informação</t>
+        </is>
+      </c>
       <c r="K155" s="3" t="inlineStr"/>
       <c r="L155" s="3" t="inlineStr"/>
       <c r="M155" s="3" t="inlineStr"/>
-      <c r="N155" s="3" t="inlineStr">
+      <c r="N155" s="3" t="inlineStr"/>
+      <c r="O155" s="3" t="inlineStr">
         <is>
           <t>https://kaiserso.github.io/INS_delphi/hiv/hiv_154.html</t>
         </is>

</xml_diff>